<commit_message>
TestData From Excel is provided
</commit_message>
<xml_diff>
--- a/RestAssured/LMS-API-Testing/src/test/resources/TestData.xlsx
+++ b/RestAssured/LMS-API-Testing/src/test/resources/TestData.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Expleo-Training\RestAssured\LMS-API-Testing\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{595E0A8D-662E-4657-9FB8-640B6E4C04D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5B5D421-9B22-43BF-80D4-31B549282BB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{FA590FFE-4008-4D37-AE77-A5C822031AC3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{FA590FFE-4008-4D37-AE77-A5C822031AC3}"/>
   </bookViews>
   <sheets>
     <sheet name="ValidLogin" sheetId="1" r:id="rId1"/>
     <sheet name="InvalidLogin" sheetId="2" r:id="rId2"/>
+    <sheet name="ValidParamsForGetAllNotes" sheetId="3" r:id="rId3"/>
+    <sheet name="InvalidParamsForGetAllNotes" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="41">
   <si>
     <t>Password</t>
   </si>
@@ -70,13 +72,103 @@
   </si>
   <si>
     <t>Invalid Email</t>
+  </si>
+  <si>
+    <t>isAuthRequired</t>
+  </si>
+  <si>
+    <t>page</t>
+  </si>
+  <si>
+    <t>limit</t>
+  </si>
+  <si>
+    <t>search</t>
+  </si>
+  <si>
+    <t>tags</t>
+  </si>
+  <si>
+    <t>isPinned</t>
+  </si>
+  <si>
+    <t>sortBy</t>
+  </si>
+  <si>
+    <t>sortOrder</t>
+  </si>
+  <si>
+    <t>title</t>
+  </si>
+  <si>
+    <t>asc</t>
+  </si>
+  <si>
+    <t>API</t>
+  </si>
+  <si>
+    <t>qa</t>
+  </si>
+  <si>
+    <t>lastEdited</t>
+  </si>
+  <si>
+    <t>desc</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>demo</t>
+  </si>
+  <si>
+    <t>expectedStatusCode</t>
+  </si>
+  <si>
+    <t>expectedMessage</t>
+  </si>
+  <si>
+    <t>Unauthorized</t>
+  </si>
+  <si>
+    <t>Invalid page number</t>
+  </si>
+  <si>
+    <t>Invalid limit</t>
+  </si>
+  <si>
+    <t>invalid</t>
+  </si>
+  <si>
+    <t>Invalid sortBy value</t>
+  </si>
+  <si>
+    <t>Invalid sortOrder value</t>
+  </si>
+  <si>
+    <t>{"$ne":null}</t>
+  </si>
+  <si>
+    <t>Invalid search parameter</t>
+  </si>
+  <si>
+    <t>@#$</t>
+  </si>
+  <si>
+    <t>Invalid tag</t>
+  </si>
+  <si>
+    <t>aaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaa</t>
+  </si>
+  <si>
+    <t>Search text too long</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -105,16 +197,33 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -122,16 +231,43 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBBBBBB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBBBBBB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -561,4 +697,538 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AED77E9F-F616-42E4-BE39-6D3DCEE08DF1}">
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5">
+        <v>1</v>
+      </c>
+      <c r="C2" s="5">
+        <v>10</v>
+      </c>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="B3" s="5">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5">
+        <v>10</v>
+      </c>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="B4" s="5">
+        <v>2</v>
+      </c>
+      <c r="C4" s="5">
+        <v>5</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5">
+        <v>1</v>
+      </c>
+      <c r="C5" s="5">
+        <v>50</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="B6" s="5">
+        <v>10</v>
+      </c>
+      <c r="C6" s="5">
+        <v>1</v>
+      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94D561FD-D60B-404D-8EB6-EF178A6DDB98}">
+  <dimension ref="A1:J13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:10" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="B2" s="7">
+        <v>1</v>
+      </c>
+      <c r="C2" s="7">
+        <v>10</v>
+      </c>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" s="7">
+        <v>401</v>
+      </c>
+      <c r="J2" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7">
+        <v>0</v>
+      </c>
+      <c r="C3" s="7">
+        <v>10</v>
+      </c>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" s="7">
+        <v>400</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="B4" s="7">
+        <v>11</v>
+      </c>
+      <c r="C4" s="7">
+        <v>10</v>
+      </c>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" s="7">
+        <v>400</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A5" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="B5" s="7">
+        <v>1</v>
+      </c>
+      <c r="C5" s="7">
+        <v>0</v>
+      </c>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="7">
+        <v>400</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="B6" s="7">
+        <v>1</v>
+      </c>
+      <c r="C6" s="7">
+        <v>51</v>
+      </c>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="7">
+        <v>400</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="B7" s="7">
+        <v>1</v>
+      </c>
+      <c r="C7" s="7">
+        <v>10</v>
+      </c>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I7" s="7">
+        <v>400</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="B8" s="7">
+        <v>1</v>
+      </c>
+      <c r="C8" s="7">
+        <v>10</v>
+      </c>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="I8" s="7">
+        <v>400</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="B9" s="7">
+        <v>1</v>
+      </c>
+      <c r="C9" s="7">
+        <v>10</v>
+      </c>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I9" s="7">
+        <v>400</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="B10" s="7">
+        <v>1</v>
+      </c>
+      <c r="C10" s="7">
+        <v>10</v>
+      </c>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7">
+        <v>400</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7">
+        <v>1</v>
+      </c>
+      <c r="C11" s="7">
+        <v>10</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I11" s="7">
+        <v>400</v>
+      </c>
+      <c r="J11" s="7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A12" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="B12" s="7">
+        <v>1</v>
+      </c>
+      <c r="C12" s="7">
+        <v>10</v>
+      </c>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F12" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I12" s="7">
+        <v>400</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="184.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="B13" s="7">
+        <v>1</v>
+      </c>
+      <c r="C13" s="7">
+        <v>10</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I13" s="7">
+        <v>400</v>
+      </c>
+      <c r="J13" s="7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Control Flow Problems Solved
</commit_message>
<xml_diff>
--- a/RestAssured/LMS-API-Testing/src/test/resources/TestData.xlsx
+++ b/RestAssured/LMS-API-Testing/src/test/resources/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Expleo-Training\RestAssured\LMS-API-Testing\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5B5D421-9B22-43BF-80D4-31B549282BB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32B306EF-1290-4490-93F1-E3AD4471F38A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{FA590FFE-4008-4D37-AE77-A5C822031AC3}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{FA590FFE-4008-4D37-AE77-A5C822031AC3}"/>
   </bookViews>
   <sheets>
     <sheet name="ValidLogin" sheetId="1" r:id="rId1"/>
@@ -158,10 +158,10 @@
     <t>Invalid tag</t>
   </si>
   <si>
-    <t>aaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaa</t>
-  </si>
-  <si>
     <t>Search text too long</t>
+  </si>
+  <si>
+    <t>dnwcjnwdddccrefjwnfeuife3ufdu32b4dfu34f8808edhwichwoichwinxei3idj3u4d9jjewdj</t>
   </si>
 </sst>
 </file>
@@ -223,7 +223,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -246,6 +246,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBBBBBB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBBBBBB"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -262,11 +273,11 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -701,7 +712,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AED77E9F-F616-42E4-BE39-6D3DCEE08DF1}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
@@ -846,6 +857,11 @@
       </c>
       <c r="H6" s="5" t="s">
         <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -859,373 +875,373 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:10" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="4" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="B2" s="7">
-        <v>1</v>
-      </c>
-      <c r="C2" s="7">
-        <v>10</v>
-      </c>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G2" s="7" t="s">
+      <c r="A2" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="B2" s="6">
+        <v>1</v>
+      </c>
+      <c r="C2" s="6">
+        <v>10</v>
+      </c>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G2" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="I2" s="7">
+      <c r="I2" s="6">
         <v>401</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="J2" s="6" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="B3" s="7">
-        <v>0</v>
-      </c>
-      <c r="C3" s="7">
-        <v>10</v>
-      </c>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G3" s="7" t="s">
+      <c r="A3" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B3" s="6">
+        <v>0</v>
+      </c>
+      <c r="C3" s="6">
+        <v>10</v>
+      </c>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G3" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="7">
+      <c r="I3" s="6">
         <v>400</v>
       </c>
-      <c r="J3" s="7" t="s">
+      <c r="J3" s="6" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="B4" s="7">
+      <c r="A4" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6">
         <v>11</v>
       </c>
-      <c r="C4" s="7">
-        <v>10</v>
-      </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G4" s="7" t="s">
+      <c r="C4" s="6">
+        <v>10</v>
+      </c>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G4" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="6">
         <v>400</v>
       </c>
-      <c r="J4" s="7" t="s">
+      <c r="J4" s="6" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="B5" s="7">
-        <v>1</v>
-      </c>
-      <c r="C5" s="7">
-        <v>0</v>
-      </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G5" s="7" t="s">
+      <c r="A5" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B5" s="6">
+        <v>1</v>
+      </c>
+      <c r="C5" s="6">
+        <v>0</v>
+      </c>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="6">
         <v>400</v>
       </c>
-      <c r="J5" s="7" t="s">
+      <c r="J5" s="6" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="B6" s="7">
-        <v>1</v>
-      </c>
-      <c r="C6" s="7">
+      <c r="A6" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B6" s="6">
+        <v>1</v>
+      </c>
+      <c r="C6" s="6">
         <v>51</v>
       </c>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G6" s="7" t="s">
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="6">
         <v>400</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="J6" s="6" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="B7" s="7">
-        <v>1</v>
-      </c>
-      <c r="C7" s="7">
-        <v>10</v>
-      </c>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G7" s="7" t="s">
+      <c r="A7" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B7" s="6">
+        <v>1</v>
+      </c>
+      <c r="C7" s="6">
+        <v>10</v>
+      </c>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G7" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="I7" s="7">
+      <c r="I7" s="6">
         <v>400</v>
       </c>
-      <c r="J7" s="7" t="s">
+      <c r="J7" s="6" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="B8" s="7">
-        <v>1</v>
-      </c>
-      <c r="C8" s="7">
-        <v>10</v>
-      </c>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G8" s="7" t="s">
+      <c r="A8" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B8" s="6">
+        <v>1</v>
+      </c>
+      <c r="C8" s="6">
+        <v>10</v>
+      </c>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G8" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="6">
         <v>400</v>
       </c>
-      <c r="J8" s="7" t="s">
+      <c r="J8" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="B9" s="7">
-        <v>1</v>
-      </c>
-      <c r="C9" s="7">
-        <v>10</v>
-      </c>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7" t="s">
+      <c r="A9" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B9" s="6">
+        <v>1</v>
+      </c>
+      <c r="C9" s="6">
+        <v>10</v>
+      </c>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="I9" s="7">
+      <c r="I9" s="6">
         <v>400</v>
       </c>
-      <c r="J9" s="7" t="s">
+      <c r="J9" s="6" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="B10" s="7">
-        <v>1</v>
-      </c>
-      <c r="C10" s="7">
-        <v>10</v>
-      </c>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G10" s="7" t="s">
+      <c r="A10" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B10" s="6">
+        <v>1</v>
+      </c>
+      <c r="C10" s="6">
+        <v>10</v>
+      </c>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G10" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7">
+      <c r="H10" s="6"/>
+      <c r="I10" s="6">
         <v>400</v>
       </c>
-      <c r="J10" s="7" t="s">
+      <c r="J10" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="B11" s="7">
-        <v>1</v>
-      </c>
-      <c r="C11" s="7">
-        <v>10</v>
-      </c>
-      <c r="D11" s="7" t="s">
+      <c r="A11" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B11" s="6">
+        <v>1</v>
+      </c>
+      <c r="C11" s="6">
+        <v>10</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G11" s="7" t="s">
+      <c r="E11" s="6"/>
+      <c r="F11" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G11" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="H11" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="6">
         <v>400</v>
       </c>
-      <c r="J11" s="7" t="s">
+      <c r="J11" s="6" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="B12" s="7">
-        <v>1</v>
-      </c>
-      <c r="C12" s="7">
-        <v>10</v>
-      </c>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7" t="s">
+      <c r="A12" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B12" s="6">
+        <v>1</v>
+      </c>
+      <c r="C12" s="6">
+        <v>10</v>
+      </c>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G12" s="7" t="s">
+      <c r="F12" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="I12" s="7">
+      <c r="I12" s="6">
         <v>400</v>
       </c>
-      <c r="J12" s="7" t="s">
+      <c r="J12" s="6" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="184.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="B13" s="7">
-        <v>1</v>
-      </c>
-      <c r="C13" s="7">
-        <v>10</v>
-      </c>
-      <c r="D13" s="7" t="s">
+    <row r="13" spans="1:10" ht="118.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B13" s="6">
+        <v>1</v>
+      </c>
+      <c r="C13" s="6">
+        <v>10</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I13" s="6">
+        <v>400</v>
+      </c>
+      <c r="J13" s="6" t="s">
         <v>39</v>
-      </c>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="I13" s="7">
-        <v>400</v>
-      </c>
-      <c r="J13" s="7" t="s">
-        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>